<commit_message>
Compute epcr with Bayesian ACMG framework instead of hand assignment
epcr = P_variant (Tavtigian point system) x P_gene (validity tier)
x P_inheritance. Adds epcr.py, epcr_audit.tsv and EPCR_METHOD.md;
methods form updated to describe the computation.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_filled.xlsx
+++ b/submission/methods_description_form_filled.xlsx
@@ -569,7 +569,7 @@
 3. Annotation: Ensembl VEP 115.2 (Docker, offline cache 115, GRCh38) with HGVS, MANE/canonical, SIFT, PolyPhen, gnomAD exome and genome allele frequencies, and ClinVar via --check_existing.
 4. Prioritisation: Exomiser 15.1.0 (data release 2512, hg38), PASS-only, removing UTR/intronic/intergenic/regulatory effects; maximum population frequency 2%, with mode-specific cutoffs of 0.1% for dominant/hom-alt and 2% for compound het; pathogenicity sources REVEL, MVP, AlphaMissense and SpliceAI; OMIM and hiPHIVE phenotype prioritisers. Exomiser scores all inheritance modes, including compound-heterozygous pairs.
 5. Targeted review: every rare (max gnomAD AF &lt;1%) MANE/canonical variant from the VEP output was screened for (a) ClinVar pathogenic/likely pathogenic, (b) HIGH/MODERATE impact in a phenotype-driven gene panel (spindle assembly checkpoint / MVA genes, rhabdomyosarcoma predisposition and RASopathy genes, nephrocalcinosis genes, primordial dwarfism and DNA repair genes) and (c) ACMG SF v3.2 genes for secondary findings.
-6. Curation and ranking: candidates were kept or dropped by genotype, read support, allele frequency, predicted effect, gene-disease fit and inheritance. Apparent compound-het pairs whose two variants lie a few bp apart (FANCD2, SERPINA1, MTCH2, ADAMTS1) were treated as cis/single events, not two hits. Recurrent artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) were excluded. Every call was checked against the VCF (PASS, genotype, allele depths). epcr is a manually assigned probability that the row is causal (primary) or a true reportable finding (secondary). Rows are listed primary first, by decreasing epcr, then secondary.</t>
+6. Curation and ranking: candidates were kept or dropped by genotype, read support, allele frequency, predicted effect, gene-disease fit and inheritance. Apparent compound-het pairs whose two variants lie a few bp apart (FANCD2, SERPINA1, MTCH2, ADAMTS1) were treated as cis/single events, not two hits. Recurrent artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) were excluded. Every call was checked against the VCF (PASS, genotype, allele depths). epcr is computed, not assigned: epcr = P_variant x P_gene x P_inheritance, where P_variant is the Bayesian ACMG posterior (Tavtigian 2018/2020 point system: prior 0.10, odds x2.08 per point; product over both variants of a pair), P_gene is a ClinGen-style gene-disease validity tier (definitive 1.0 ... none 0.02) and P_inheritance is the probability the inheritance requirement is met (trans phase for a pair, second-hit chance for a lone het in a recessive gene, penetrance for a dominant secondary finding). Every ACMG criterion and constant is listed per row in epcr.py and epcr_audit.tsv. Rows are listed primary first, by decreasing epcr, then secondary.</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Manual review of the Exomiser ranking and filtered VEP candidates: (1) removed artefact-prone loci (HLA class I/II, MUC4, KRTAP, olfactory receptors); (2) re-evaluated Exomiser compound-het calls and rejected pairs whose variants lie within a few bp (likely the same haplotype/complex event); (3) checked gene-disease fit against the phenotype using OMIM/ClinVar knowledge (BUB1B biallelic loss -&gt; mosaic variegated aneuploidy type 1 with rhabdomyosarcoma and growth failure); (4) confirmed every submitted variant in the VCF (PASS, 0/1, allele depths about 50%); (5) assigned epcr values by hand and separated primary from secondary findings. Rows 5-7 are the next-best non-artefact Exomiser candidates, kept at low epcr to complete the top 10.</t>
+          <t>Manual review of the Exomiser ranking and filtered VEP candidates: (1) removed artefact-prone loci (HLA class I/II, MUC4, KRTAP, olfactory receptors); (2) re-evaluated Exomiser compound-het calls and rejected pairs whose variants lie within a few bp (likely the same haplotype/complex event); (3) checked gene-disease fit against the phenotype using OMIM/ClinVar knowledge (BUB1B biallelic loss -&gt; mosaic variegated aneuploidy type 1 with rhabdomyosarcoma and growth failure); (4) confirmed every submitted variant in the VCF (PASS, 0/1, allele depths about 50%); (5) assigned ACMG/AMP criteria, gene-disease validity tiers and inheritance/penetrance assumptions per row (the judgement step), from which epcr is then computed by epcr.py; separated primary from secondary findings. Rows 5-7 are the next-best non-artefact Exomiser candidates, kept at low epcr to complete the top 10.</t>
         </is>
       </c>
     </row>
@@ -690,10 +690,10 @@
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>We ranked candidate variants for a single proband with short-read whole-genome sequencing and a phenotype of rhabdomyosarcoma, nephrocalcinosis, short stature, failure to thrive, muscle atrophy, prematurity/small for gestational age and a family history of recurrent miscarriage. The pipeline pairs standard open-source tools with targeted expert-style curation.
-Methods. The VCF (GRCh38) was annotated with Ensembl VEP 115 (MANE/canonical transcripts, HGVS, SIFT, PolyPhen-2, gnomAD v4 exome/genome frequencies, ClinVar). Genes were prioritised with Exomiser 15.1.0 (data release 2512) using the eight HPO terms, PASS-only calls, coding/splice effects, inheritance-specific frequency cutoffs, REVEL/MVP/AlphaMissense/SpliceAI pathogenicity and the OMIM and hiPHIVE phenotype prioritisers. Rare variants (&lt;1% in gnomAD) were then screened for ClinVar pathogenic calls, for HIGH/MODERATE impact in phenotype-driven gene panels (spindle assembly checkpoint/MVA, rhabdomyosarcoma predisposition and RASopathy, nephrocalcinosis, growth/DNA repair) and in ACMG SF v3.2 genes. Candidates were curated for genotype quality, allele balance, frequency, predicted effect, gene-disease fit and inheritance plausibility. A manually assigned epcr reflects our estimated probability of causality.
-Result. The top candidate is a presumed compound-heterozygous pair in BUB1B: c.2210T&gt;G p.(Leu737*) (ClinVar pathogenic/likely pathogenic, gnomAD 7.9e-05) and c.3006T&gt;G p.(Asn1002Lys), a novel missense in the kinase domain (absent from gnomAD, AlphaMissense 0.92, SIFT deleterious, PolyPhen 0.997). Both are high-quality heterozygous PASS calls with balanced allele depths. Biallelic BUB1B loss causes mosaic variegated aneuploidy type 1 (MVA1), which fits the embryonal rhabdomyosarcoma, pre- and postnatal growth failure and the reproductive history. A truncating allele plus a hypomorphic kinase-domain missense is the classic MVA1 genotype. Exomiser ranked BUB1B first (p = 0.0005, ~30-fold ahead of the next gene). Lower-ranked primary rows include a possible nephrocalcinosis contributor (SLC34A1 p.Ala133Val), a same-pathway heterozygous variant (MAD1L1 p.Arg59Cys) and the best remaining Exomiser candidates. Three heterozygous P/LP variants unrelated to the phenotype are reported as secondary findings (LZTR1, GNRHR, FLG).
-Strengths. Uses only public data and open-source tools and is reproducible on a laptop. It combines phenotype-driven whole-genome ranking with curation that removes common false positives: artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) and pseudo-compound-het pairs whose variants lie a few bp apart and are almost certainly in cis. Compound-heterozygous pairs are output natively. Every submitted variant was checked in the VCF.
-Limitations. Singleton data: the BUB1B variants are ~11 kb apart, so trans phase cannot be established from short reads. Parental testing or long-read sequencing is needed. The missense allele has no functional data. Structural variants, copy-number changes, repeat expansions, mitochondrial and deep-intronic/regulatory variants were not systematically assessed, since the Exomiser run excluded intronic/UTR effects. The ranking depends on curated knowledge and manually assigned epcr values, so it is not fully automated. Lower-ranked rows have low prior probability and mainly complete the top-10 list. A bulk-WGS screen (GC-corrected depth and allele-balance per chromosome, centromeres masked) found no clonal whole-chromosome gain or loss, but variegated aneuploidy averages out in bulk data, so this neither supports nor refutes MVA; karyotyping is needed.</t>
+Methods. The VCF (GRCh38) was annotated with Ensembl VEP 115 (MANE/canonical transcripts, HGVS, SIFT, PolyPhen-2, gnomAD v4 exome/genome frequencies, ClinVar). Genes were prioritised with Exomiser 15.1.0 (data release 2512) using the eight HPO terms, PASS-only calls, coding/splice effects, inheritance-specific frequency cutoffs, REVEL/MVP/AlphaMissense/SpliceAI pathogenicity and the OMIM and hiPHIVE phenotype prioritisers. Rare variants (&lt;1% in gnomAD) were then screened for ClinVar pathogenic calls, for HIGH/MODERATE impact in phenotype-driven gene panels (MVA/spindle checkpoint, rhabdomyosarcoma predisposition, nephrocalcinosis, growth/DNA repair) and in ACMG SF v3.2 genes. Candidates were curated for genotype quality, allele balance, frequency, predicted effect, gene-disease fit and inheritance plausibility. epcr is computed as P(variant pathogenic) x P(gene causes phenotype) x P(inheritance met), with the first term from the Bayesian ACMG point system (Tavtigian 2020), so each value can be audited criterion by criterion.
+Result. The top candidate is a presumed compound-heterozygous pair in BUB1B: c.2210T&gt;G p.(Leu737*) (ClinVar pathogenic/likely pathogenic, gnomAD 7.9e-05) and c.3006T&gt;G p.(Asn1002Lys), a novel missense in the kinase domain (absent from gnomAD, AlphaMissense 0.92, SIFT deleterious, PolyPhen 0.997). Biallelic BUB1B loss causes mosaic variegated aneuploidy type 1 (MVA1), which fits the embryonal rhabdomyosarcoma, pre- and postnatal growth failure and the reproductive history. A truncating allele plus a hypomorphic kinase-domain missense is the classic MVA1 genotype. Exomiser ranked BUB1B first (p = 0.0005, ~30-fold ahead of the next gene). Computed epcr for the pair is 0.72: the truncating allele scores as pathogenic (0.99) but the novel missense reaches only 0.81 under strict ACMG scoring, and trans phase is unproven (0.9). Lower-ranked primary rows include a possible nephrocalcinosis contributor (SLC34A1 p.Ala133Val), a same-pathway heterozygous variant (MAD1L1 p.Arg59Cys) and the best remaining Exomiser candidates. Three heterozygous P/LP variants unrelated to the phenotype are reported as secondary findings (LZTR1, GNRHR, FLG).
+Strengths. Uses only public data and open-source tools and is reproducible on a laptop. It combines phenotype-driven whole-genome ranking with curation that removes common false positives: artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) and pseudo-compound-het pairs whose variants lie a few bp apart and are almost certainly in cis. Compound-heterozygous pairs are output natively.
+Limitations. Singleton data: the BUB1B variants are ~11 kb apart, so trans phase cannot be established from short reads. Parental testing or long-read sequencing is needed. The missense allele has no functional data. Structural, copy-number, repeat-expansion, mitochondrial and deep-intronic/regulatory variants were not systematically assessed. Assigning ACMG criteria, validity tiers and penetrance values is still a curated step, so the pipeline is not fully automated. Lower-ranked rows have low computed probability and mainly complete the top-10 list. A bulk-WGS screen (GC-corrected depth and allele-balance per chromosome, centromeres masked) found no clonal whole-chromosome gain or loss, but variegated aneuploidy averages out in bulk data, so this neither supports nor refutes MVA; karyotyping is needed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Methods form: add whole-genome Exomiser rerun (SpliceAI, no REMM yet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_filled.xlsx
+++ b/submission/methods_description_form_filled.xlsx
@@ -567,7 +567,7 @@
           <t>1. Input: proband short-read WGS VCF (WGS_EX2312012, GRCh38, singleton, no parental data) and the 8 HPO terms from the clinical phenotype (HP:0002859, HP:0000121, HP:0004322, HP:0001508, HP:0003202, HP:0001622, HP:0001518, HP:0200067).
 2. QC: per-chromosome depth, B-allele-frequency histogram, runs of homozygosity (bcftools roh) and 1 Mb read-depth bins from a re-aligned read subsample (minimap2 2.31). Sex verified as male from X/Y genotypes. Bulk aneuploidy screen: per-chromosome GC-corrected depth ratio (1.00 on all autosomes) and B-allele-frequency deviation of heterozygous PASS SNPs with centromeric/acrocentric windows masked (6-8% off-centre on every autosome). No clonal whole-chromosome gain or loss is detectable in blood WGS; note that variegated (cell-to-cell random) aneuploidy averages out in bulk sequencing and is not expected to be visible here. Used as sanity checks; not used to score variants.
 3. Annotation: Ensembl VEP 115.2 (Docker, offline cache 115, GRCh38) with HGVS, MANE/canonical, SIFT, PolyPhen, gnomAD exome and genome allele frequencies, and ClinVar via --check_existing.
-4. Prioritisation: Exomiser 15.1.0 (data release 2512, hg38), PASS-only, removing UTR/intronic/intergenic/regulatory effects; maximum population frequency 2%, with mode-specific cutoffs of 0.1% for dominant/hom-alt and 2% for compound het; pathogenicity sources REVEL, MVP, AlphaMissense and SpliceAI; OMIM and hiPHIVE phenotype prioritisers. Exomiser scores all inheritance modes, including compound-heterozygous pairs.
+4. Prioritisation: Exomiser 15.1.0 (data release 2512, hg38), PASS-only, removing UTR/intronic/intergenic/regulatory effects; maximum population frequency 2%, with mode-specific cutoffs of 0.1% for dominant/hom-alt and 2% for compound het; pathogenicity sources REVEL, MVP, AlphaMissense and SpliceAI; OMIM and hiPHIVE phenotype prioritisers. Exomiser scores all inheritance modes, including compound-heterozygous pairs. A second, whole-genome Exomiser run (following the official preset-genome-analysis model, analysis/proband_genome.yml) additionally kept intronic, UTR and regulatory-region variants, applied Exomiser's allele-balance filter and scored non-coding variants with SpliceAI; REMM regulatory scores were not yet available. This run left the top of the ranking unchanged (BUB1B first, p = 0.0004), and found no intronic/splice-altering variant in BUB1B, CEP57 or TRIP13 and no non-coding variant with SpliceAI &gt;= 0.5 anywhere in the prioritised genes.
 5. Targeted review: every rare (max gnomAD AF &lt;1%) MANE/canonical variant from the VEP output was screened for (a) ClinVar pathogenic/likely pathogenic, (b) HIGH/MODERATE impact in a phenotype-driven gene panel (spindle assembly checkpoint / MVA genes, rhabdomyosarcoma predisposition and RASopathy genes, nephrocalcinosis genes, primordial dwarfism and DNA repair genes) and (c) ACMG SF v3.2 genes for secondary findings.
 6. Curation and ranking: candidates were kept or dropped by genotype, read support, allele frequency, predicted effect, gene-disease fit and inheritance. Apparent compound-het pairs whose two variants lie a few bp apart (FANCD2, SERPINA1, MTCH2, ADAMTS1) were treated as cis/single events, not two hits. Recurrent artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) were excluded. Every call was checked against the VCF (PASS, genotype, allele depths). epcr is computed, not assigned: epcr = P_variant x P_gene x P_inheritance, where P_variant is the Bayesian ACMG posterior (Tavtigian 2018/2020 point system: prior 0.10, odds x2.08 per point; product over both variants of a pair), P_gene is a ClinGen-style gene-disease validity tier (definitive 1.0 ... none 0.02) and P_inheritance is the probability the inheritance requirement is met (trans phase for a pair, second-hit chance for a lone het in a recessive gene, penetrance for a dominant secondary finding). Every ACMG criterion and constant is listed per row in epcr.py and epcr_audit.tsv. Rows are listed primary first, by decreasing epcr, then secondary.</t>
         </is>
@@ -689,11 +689,11 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>We ranked candidate variants for a single proband with short-read whole-genome sequencing and a phenotype of rhabdomyosarcoma, nephrocalcinosis, short stature, failure to thrive, muscle atrophy, prematurity/small for gestational age and a family history of recurrent miscarriage. The pipeline pairs standard open-source tools with targeted expert-style curation.
+          <t>We ranked candidate variants for a single proband with short-read whole-genome sequencing and a phenotype of rhabdomyosarcoma, nephrocalcinosis, short stature, failure to thrive, muscle atrophy, prematurity/small for gestational age and a family history of recurrent miscarriage. We pair standard open-source tools with targeted curation.
 Methods. The VCF (GRCh38) was annotated with Ensembl VEP 115 (MANE/canonical transcripts, HGVS, SIFT, PolyPhen-2, gnomAD v4 exome/genome frequencies, ClinVar). Genes were prioritised with Exomiser 15.1.0 (data release 2512) using the eight HPO terms, PASS-only calls, coding/splice effects, inheritance-specific frequency cutoffs, REVEL/MVP/AlphaMissense/SpliceAI pathogenicity and the OMIM and hiPHIVE phenotype prioritisers. Rare variants (&lt;1% in gnomAD) were then screened for ClinVar pathogenic calls, for HIGH/MODERATE impact in phenotype-driven gene panels (MVA/spindle checkpoint, rhabdomyosarcoma predisposition, nephrocalcinosis, growth/DNA repair) and in ACMG SF v3.2 genes. Candidates were curated for genotype quality, allele balance, frequency, predicted effect, gene-disease fit and inheritance plausibility. epcr is computed as P(variant pathogenic) x P(gene causes phenotype) x P(inheritance met), with the first term from the Bayesian ACMG point system (Tavtigian 2020), so each value can be audited criterion by criterion.
 Result. The top candidate is a presumed compound-heterozygous pair in BUB1B: c.2210T&gt;G p.(Leu737*) (ClinVar pathogenic/likely pathogenic, gnomAD 7.9e-05) and c.3006T&gt;G p.(Asn1002Lys), a novel missense in the kinase domain (absent from gnomAD, AlphaMissense 0.92, SIFT deleterious, PolyPhen 0.997). Biallelic BUB1B loss causes mosaic variegated aneuploidy type 1 (MVA1), which fits the embryonal rhabdomyosarcoma, pre- and postnatal growth failure and the reproductive history. A truncating allele plus a hypomorphic kinase-domain missense is the classic MVA1 genotype. Exomiser ranked BUB1B first (p = 0.0005, ~30-fold ahead of the next gene). Computed epcr for the pair is 0.72: the truncating allele scores as pathogenic (0.99) but the novel missense reaches only 0.81 under strict ACMG scoring, and trans phase is unproven (0.9). Lower-ranked primary rows include a possible nephrocalcinosis contributor (SLC34A1 p.Ala133Val), a same-pathway heterozygous variant (MAD1L1 p.Arg59Cys) and the best remaining Exomiser candidates. Three heterozygous P/LP variants unrelated to the phenotype are reported as secondary findings (LZTR1, GNRHR, FLG).
-Strengths. Uses only public data and open-source tools and is reproducible on a laptop. It combines phenotype-driven whole-genome ranking with curation that removes common false positives: artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) and pseudo-compound-het pairs whose variants lie a few bp apart and are almost certainly in cis. Compound-heterozygous pairs are output natively.
-Limitations. Singleton data: the BUB1B variants are ~11 kb apart, so trans phase cannot be established from short reads. Parental testing or long-read sequencing is needed. The missense allele has no functional data. Structural, copy-number, repeat-expansion, mitochondrial and deep-intronic/regulatory variants were not systematically assessed. Assigning ACMG criteria, validity tiers and penetrance values is still a curated step, so the pipeline is not fully automated. Lower-ranked rows have low computed probability and mainly complete the top-10 list. A bulk-WGS screen (GC-corrected depth and allele-balance per chromosome, centromeres masked) found no clonal whole-chromosome gain or loss, but variegated aneuploidy averages out in bulk data, so this neither supports nor refutes MVA; karyotyping is needed.</t>
+Strengths. Public data and open-source tools only; reproducible on a laptop. Combines phenotype-driven whole-genome ranking with curation that removes common false positives: artefact-prone loci (HLA, MUC4, KRTAP, olfactory receptors) and pseudo-compound-het pairs whose variants lie a few bp apart and are almost certainly in cis. Compound-heterozygous pairs are output natively.
+Limitations. Singleton data: the BUB1B variants are ~11 kb apart, so trans phase cannot be established from short reads. Parental testing or long-read sequencing is needed. The missense allele has no functional data. A whole-genome rerun scoring intronic variants with SpliceAI kept BUB1B first; structural, copy-number, repeat-expansion, mitochondrial and purely regulatory variants were not assessed. Assigning ACMG criteria, validity tiers and penetrance values is still a curated step, so the pipeline is not fully automated. Lower-ranked rows mainly complete the top-10 list. A bulk-WGS screen (GC-corrected depth and allele-balance per chromosome, centromeres masked) found no clonal whole-chromosome gain or loss, but variegated aneuploidy averages out in bulk data, so this neither supports nor refutes MVA; karyotyping is needed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final Track 1 submission (team semel): report, ranked CSV, full pipeline scripts
Adds the submitted predictions file and report, the REMM/LIRICAL/SV pipeline
scripts and Exomiser configs, a README, and a .gitignore that keeps all
patient data and derived files out of the repository.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_filled.xlsx
+++ b/submission/methods_description_form_filled.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>[TODO: team name]</t>
+          <t>semel</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Anthropic Claude Code CLI, model Claude Opus 5.5, [TODO: plan/tier, e.g. Claude Max / Team / API], [TODO: data setting, e.g. commercial terms, no training on customer content]. Used as a coding and analysis assistant (writing pipeline scripts, querying annotation output, drafting curation notes and this form). All variant calls and final rankings were checked against the underlying VCF and annotations.</t>
+          <t>Anthropic Claude Code CLI, model Claude Opus 5.5, Claude Max plan, training opt-out enabled, no feedback provided. Used as a coding and analysis assistant (writing pipeline scripts, querying annotation output, drafting curation notes and this form). All variant calls and final rankings were checked against the underlying VCF and annotations.</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Manual review of the Exomiser ranking and filtered VEP candidates: (1) removed artefact-prone loci (HLA class I/II, MUC4, KRTAP, olfactory receptors); (2) re-evaluated Exomiser compound-het calls and rejected pairs whose variants lie within a few bp (likely the same haplotype/complex event); (3) checked gene-disease fit against the phenotype using OMIM/ClinVar knowledge (BUB1B biallelic loss -&gt; mosaic variegated aneuploidy type 1 with rhabdomyosarcoma and growth failure); (4) confirmed every submitted variant in the VCF (PASS, 0/1, allele depths about 50%); (5) assigned ACMG/AMP criteria, gene-disease validity tiers and inheritance/penetrance assumptions per row (the judgement step), from which epcr is then computed by epcr.py; separated primary from secondary findings. Rows 5-7 are the next-best non-artefact Exomiser candidates, kept at low epcr to complete the top 10.</t>
+          <t>Manual review of the Exomiser ranking and filtered VEP candidates: (1) removed artefact-prone loci (HLA class I/II, MUC4, KRTAP, olfactory receptors); (2) re-evaluated Exomiser compound-het calls and rejected pairs whose variants lie within a few bp (likely the same haplotype/complex event); (3) checked gene-disease fit against the phenotype using OMIM/ClinVar knowledge (BUB1B biallelic loss -&gt; mosaic variegated aneuploidy type 1 with rhabdomyosarcoma and growth failure); (4) confirmed every submitted variant in the VCF (PASS, 0/1, allele depths checked; SLC34A1 and FANCD2 sit near 30%); (5) assigned ACMG/AMP criteria, gene-disease validity tiers and inheritance/penetrance assumptions per row (the judgement step), from which epcr is then computed by epcr.py; separated primary from secondary findings. Rows 5-7 are the next-best non-artefact Exomiser candidates, kept at low epcr to complete the top 10.</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Local laptop (Apple M2 Max, 12 cores, 32 GB RAM); no cloud cost. Exomiser: ~42 s after data unpacking. VEP whole-genome annotation of ~5.0 M records: 36 h 38 min wall time (VEP stats: 131,888 s; Docker Desktop on macOS, --fork 10, --hgvs against a gzipped FASTA). This was an unoptimised single-process run; splitting the VCF per chromosome, running VEP natively with an uncompressed indexed FASTA and dropping --hgvs would reduce it to a few hours, and Exomiser alone gives the same top gene in under a minute. An earlier VEP attempt with --everything was abandoned after ~3 h. Data/cache downloads: several hours. Manual curation and review: ~[TODO: hours] person-hours.</t>
+          <t>Local laptop (Apple M2 Max, 12 cores, 32 GB RAM); no cloud cost. Exomiser: ~42 s after data unpacking. VEP whole-genome annotation of ~5.0 M records: 36 h 38 min wall time (VEP stats: 131,888 s; Docker Desktop on macOS, --fork 10, --hgvs against a gzipped FASTA). This was an unoptimised single-process run; splitting the VCF per chromosome, running VEP natively with an uncompressed indexed FASTA and dropping --hgvs would reduce it to a few hours, and Exomiser alone gives the same top gene in under a minute. An earlier VEP attempt with --everything was abandoned after ~3 h. Data/cache downloads: several hours. Manual curation and review: not formally tracked.</t>
         </is>
       </c>
     </row>

</xml_diff>